<commit_message>
update data publication lags
Applied shift_by_vector lags across all blocks based on guidelines
</commit_message>
<xml_diff>
--- a/shift_report.xlsx
+++ b/shift_report.xlsx
@@ -7,12 +7,21 @@
   </bookViews>
   <sheets>
     <sheet name="FX_liqudity" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="personal_labor_income_taxes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="corporate_business_tax" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="consumption_tax" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="import_trade_tax" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="real_estate" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="real_activity" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="capital_markets" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="labor" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="adjusters" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
   <si>
     <t xml:space="preserve">variable</t>
   </si>
@@ -27,6 +36,174 @@
   </si>
   <si>
     <t xml:space="preserve">Foreign exchange reserves (millions of dollars)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Gross Income Tax Division</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total refunds from the Income Tax Department</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Income Tax Division Net</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deductions and the capital market</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deduction from salary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Independents advances</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Self-employed tax differences</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Independent Cancellations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">self employed returns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capital Gains Tax Refunds</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VAT Financial Institutions (Salary)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non-profit institution tax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Companies advances</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tax differential companies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cancellation companies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Income tax for self-employed individuals and companies (advances and deductions)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Companies returns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">excess expenses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bonds and dividends</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cancellations Deductions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Goods and services</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gross local VAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VAT refund autonomy and traders</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total net VAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Net local sales tax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gross fuel tax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gross import VAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Net customs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Net import purchase tax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total import taxes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real estate taxation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Property tax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">praise tax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real estate purchase tax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">praise tax returns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">purchase returns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apartments sold at an annual rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apartment Price Index (1993=100) - Mid-period reviewed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cons_trust</t>
+  </si>
+  <si>
+    <t xml:space="preserve">madad meshulav</t>
+  </si>
+  <si>
+    <t xml:space="preserve">madad_cc_purchases_sa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">madad_pedio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">madad_yetzur_industrial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">madad_hadash</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TA35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TA125</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nasdaq</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sp500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">real salary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">salaried jobs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">unemployment rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">participation rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">employment rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VAT_rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPI</t>
   </si>
 </sst>
 </file>
@@ -368,7 +545,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -384,7 +561,626 @@
         <v>4</v>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>